<commit_message>
update MSK_bulkRNAseq_ISL1_OE results from fitting DESeq2 only using control samples for KO vs control analysis
</commit_message>
<xml_diff>
--- a/meta_data_web_portal/DAV_input_2026_01_MSK_bulkRNAseq_ISL1_OE.xlsx
+++ b/meta_data_web_portal/DAV_input_2026_01_MSK_bulkRNAseq_ISL1_OE.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="135">
   <si>
     <t xml:space="preserve">DAV</t>
   </si>
@@ -255,6 +255,9 @@
   </si>
   <si>
     <t xml:space="preserve">figures/2026_01_MSK_bulkRNAseq_ISL1_OE/volcano_plots/control_ISL1_KO_KO_vs_WT_volcano.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve">step2_DE_testing_2026_01_MSK_ISL1_OE_control.Rmd</t>
   </si>
   <si>
     <t xml:space="preserve">HGNC:8620</t>
@@ -1240,7 +1243,7 @@
         <v>79</v>
       </c>
       <c r="AA6" t="s">
-        <v>50</v>
+        <v>80</v>
       </c>
     </row>
     <row r="7">
@@ -1257,10 +1260,10 @@
         <v>30</v>
       </c>
       <c r="E7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G7" t="s">
         <v>33</v>
@@ -1305,25 +1308,25 @@
         <v>44</v>
       </c>
       <c r="U7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="V7" t="s">
         <v>35</v>
       </c>
       <c r="W7" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="X7" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Y7" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="Z7" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="AA7" t="s">
-        <v>50</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8">
@@ -1340,10 +1343,10 @@
         <v>30</v>
       </c>
       <c r="E8" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F8" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G8" t="s">
         <v>33</v>
@@ -1388,25 +1391,25 @@
         <v>44</v>
       </c>
       <c r="U8" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="V8" t="s">
         <v>35</v>
       </c>
       <c r="W8" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="X8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Y8" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Z8" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="AA8" t="s">
-        <v>50</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9">
@@ -1432,10 +1435,10 @@
         <v>33</v>
       </c>
       <c r="H9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I9" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="J9" t="s">
         <v>35</v>
@@ -1471,7 +1474,7 @@
         <v>44</v>
       </c>
       <c r="U9" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="V9" t="s">
         <v>35</v>
@@ -1480,16 +1483,16 @@
         <v>35</v>
       </c>
       <c r="X9" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="Y9" t="s">
         <v>35</v>
       </c>
       <c r="Z9" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="AA9" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10">
@@ -1515,10 +1518,10 @@
         <v>33</v>
       </c>
       <c r="H10" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J10" t="s">
         <v>35</v>
@@ -1554,7 +1557,7 @@
         <v>44</v>
       </c>
       <c r="U10" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="V10" t="s">
         <v>35</v>
@@ -1563,16 +1566,16 @@
         <v>35</v>
       </c>
       <c r="X10" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="Y10" t="s">
         <v>35</v>
       </c>
       <c r="Z10" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AA10" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11">
@@ -1598,10 +1601,10 @@
         <v>33</v>
       </c>
       <c r="H11" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I11" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="J11" t="s">
         <v>35</v>
@@ -1637,7 +1640,7 @@
         <v>44</v>
       </c>
       <c r="U11" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="V11" t="s">
         <v>35</v>
@@ -1646,16 +1649,16 @@
         <v>35</v>
       </c>
       <c r="X11" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Y11" t="s">
         <v>35</v>
       </c>
       <c r="Z11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="AA11" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12">
@@ -1681,10 +1684,10 @@
         <v>33</v>
       </c>
       <c r="H12" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I12" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J12" t="s">
         <v>35</v>
@@ -1720,7 +1723,7 @@
         <v>44</v>
       </c>
       <c r="U12" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="V12" t="s">
         <v>35</v>
@@ -1729,16 +1732,16 @@
         <v>35</v>
       </c>
       <c r="X12" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="Y12" t="s">
         <v>35</v>
       </c>
       <c r="Z12" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="AA12" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13">
@@ -1755,19 +1758,19 @@
         <v>30</v>
       </c>
       <c r="E13" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F13" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G13" t="s">
         <v>33</v>
       </c>
       <c r="H13" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I13" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="J13" t="s">
         <v>35</v>
@@ -1803,7 +1806,7 @@
         <v>44</v>
       </c>
       <c r="U13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="V13" t="s">
         <v>35</v>
@@ -1812,16 +1815,16 @@
         <v>35</v>
       </c>
       <c r="X13" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="Y13" t="s">
         <v>35</v>
       </c>
       <c r="Z13" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="AA13" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14">
@@ -1838,19 +1841,19 @@
         <v>30</v>
       </c>
       <c r="E14" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F14" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G14" t="s">
         <v>33</v>
       </c>
       <c r="H14" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J14" t="s">
         <v>35</v>
@@ -1886,7 +1889,7 @@
         <v>44</v>
       </c>
       <c r="U14" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="V14" t="s">
         <v>35</v>
@@ -1895,16 +1898,16 @@
         <v>35</v>
       </c>
       <c r="X14" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="Y14" t="s">
         <v>35</v>
       </c>
       <c r="Z14" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="AA14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15">
@@ -1930,10 +1933,10 @@
         <v>33</v>
       </c>
       <c r="H15" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I15" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="J15" t="s">
         <v>35</v>
@@ -1969,7 +1972,7 @@
         <v>44</v>
       </c>
       <c r="U15" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="V15" t="s">
         <v>35</v>
@@ -1978,16 +1981,16 @@
         <v>35</v>
       </c>
       <c r="X15" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="Y15" t="s">
         <v>35</v>
       </c>
       <c r="Z15" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AA15" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16">
@@ -2013,10 +2016,10 @@
         <v>33</v>
       </c>
       <c r="H16" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I16" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J16" t="s">
         <v>35</v>
@@ -2052,7 +2055,7 @@
         <v>44</v>
       </c>
       <c r="U16" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="V16" t="s">
         <v>35</v>
@@ -2061,16 +2064,16 @@
         <v>35</v>
       </c>
       <c r="X16" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="Y16" t="s">
         <v>35</v>
       </c>
       <c r="Z16" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="AA16" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="17">
@@ -2087,19 +2090,19 @@
         <v>30</v>
       </c>
       <c r="E17" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F17" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G17" t="s">
         <v>33</v>
       </c>
       <c r="H17" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I17" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="J17" t="s">
         <v>35</v>
@@ -2135,7 +2138,7 @@
         <v>44</v>
       </c>
       <c r="U17" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="V17" t="s">
         <v>35</v>
@@ -2144,16 +2147,16 @@
         <v>35</v>
       </c>
       <c r="X17" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="Y17" t="s">
         <v>35</v>
       </c>
       <c r="Z17" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="AA17" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="18">
@@ -2170,19 +2173,19 @@
         <v>30</v>
       </c>
       <c r="E18" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F18" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G18" t="s">
         <v>33</v>
       </c>
       <c r="H18" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I18" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J18" t="s">
         <v>35</v>
@@ -2218,7 +2221,7 @@
         <v>44</v>
       </c>
       <c r="U18" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="V18" t="s">
         <v>35</v>
@@ -2227,16 +2230,16 @@
         <v>35</v>
       </c>
       <c r="X18" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="Y18" t="s">
         <v>35</v>
       </c>
       <c r="Z18" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="AA18" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="19">
@@ -2262,10 +2265,10 @@
         <v>33</v>
       </c>
       <c r="H19" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I19" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="J19" t="s">
         <v>35</v>
@@ -2301,7 +2304,7 @@
         <v>44</v>
       </c>
       <c r="U19" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="V19" t="s">
         <v>35</v>
@@ -2310,16 +2313,16 @@
         <v>35</v>
       </c>
       <c r="X19" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="Y19" t="s">
         <v>35</v>
       </c>
       <c r="Z19" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="AA19" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="20">
@@ -2345,10 +2348,10 @@
         <v>33</v>
       </c>
       <c r="H20" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I20" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J20" t="s">
         <v>35</v>
@@ -2384,7 +2387,7 @@
         <v>44</v>
       </c>
       <c r="U20" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="V20" t="s">
         <v>35</v>
@@ -2393,16 +2396,16 @@
         <v>35</v>
       </c>
       <c r="X20" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="Y20" t="s">
         <v>35</v>
       </c>
       <c r="Z20" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="AA20" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>